<commit_message>
feat: implement KGeoMIP Analytics Framework with Streamlit interface, including configuration, monitoring, and dashboard functionalities
</commit_message>
<xml_diff>
--- a/GeoMIP/results/resultados_Geometric.xlsx
+++ b/GeoMIP/results/resultados_Geometric.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,16 @@
           <t>Tiempo de ejecución (s)</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Método</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -464,37 +474,45 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Alcance=(A,C,F,G,H,I,J,L,M) / (B,D,E,K,N,O); Mecanismo=(a,c,f,g,h,i,j,l,m) / (b,d,e,k,n,o)</t>
+          <t>Alcance=(A,B) / (C); Mecanismo=(a,b) / (c)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0,3910316228866577</t>
+          <t>1,0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0,34896183013916016</t>
+          <t>2,0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0,7399934530258179</t>
+          <t>3,0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1,0292792320251465</t>
+          <t>10,143476724624634</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -504,37 +522,45 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Alcance=(A,C,F,G,H,I,J,L,M) / (B,D,E,K,N,O); Mecanismo=(a,c,f,g,h,i,j,l,m) / (b,d,e,k,n,o)</t>
+          <t>Alcance=(A,B) / (C); Mecanismo=(a,b) / (∅)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0,3910316228866577</t>
+          <t>0,5</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0,34896183013916016</t>
+          <t>1,0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0,7399934530258179</t>
+          <t>1,5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1,0222885608673096</t>
+          <t>0,4616093635559082</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -544,37 +570,45 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Alcance=(A,B,D,E,F,H,J,K,N,O) / (C,G,I,L,M); Mecanismo=(b,d,e,f,h,j,k,n,o) / (c,g,i,l,m)</t>
+          <t>Alcance=(A,B) / (C); Mecanismo=(b) / (c)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0,3207746744155884</t>
+          <t>0,75</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0,2927582859992981</t>
+          <t>1,0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0,6135329604148865</t>
+          <t>1,75</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0,8346667289733887</t>
+          <t>0,5474703311920166</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -584,37 +618,45 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>010</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Alcance=(A,B,D,E,F,H,J,K,N,O) / (C,G,I,L,M); Mecanismo=(b,d,e,f,h,j,k,n,o) / (c,g,i,l,m)</t>
+          <t>Alcance=(A,C) / (B); Mecanismo=(∅) / (b)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0,3207746744155884</t>
+          <t>0,25</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0,2927582859992981</t>
+          <t>0,875</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0,6135329604148865</t>
+          <t>1,125</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0,9401998519897461</t>
+          <t>0,757519006729126</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -624,37 +666,45 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Alcance=(A,C,D,E,G,N,O) / (B,F,H,I,J,K,L,M); Mecanismo=(a,c,e,g,o) / (i,k,m)</t>
+          <t>Alcance=(A,C) / (B); Mecanismo=(a,c) / (∅)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0,13328880071640015</t>
+          <t>0,25</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0,15511643886566162</t>
+          <t>0,375</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0,28840523958206177</t>
+          <t>0,625</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0,8011975288391113</t>
+          <t>0,5507714748382568</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -664,37 +714,45 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>111</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Alcance=(A,B,C,D,E,F,H,J,K,N,O) / (G,I,L,M); Mecanismo=(b,d,f,h,j,n) / (l)</t>
+          <t>Alcance=(A,B) / (∅); Mecanismo=(a,b) / (c)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0,08599138259887695</t>
+          <t>0,5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0,17331552505493164</t>
+          <t>0,5</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0,2593069076538086</t>
+          <t>1,0</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0,8374013900756836</t>
+          <t>0,5224704742431641</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -704,37 +762,45 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Alcance=(A,C,D,E,F,J,N,O) / (B,G,H,I,K,L,M); Mecanismo=(a,d,e,j,n) / (b,g,h,k,m)</t>
+          <t>Alcance=(A) / (B); Mecanismo=(a) / (b)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0,11597198247909546</t>
+          <t>0,5</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0,883470356464386</t>
+          <t>0,375</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0,9994423389434814</t>
+          <t>0,875</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0,8449645042419434</t>
+          <t>0,531280517578125</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -744,37 +810,45 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>011</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Alcance=(A,C,F,G,H,I,J,L,M) / (B,D,E,K,N,O); Mecanismo=(a,c,f,g,h,i,j,l,m) / (b,d,e,k,n,o)</t>
+          <t>Alcance=(A,B) / (∅); Mecanismo=(b) / (c)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0,3910316228866577</t>
+          <t>0,75</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0,34896183013916016</t>
+          <t>0,25</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0,7399934530258179</t>
+          <t>1,0</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1,04608154296875</t>
+          <t>0,4569854736328125</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -784,37 +858,45 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>010</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Alcance=(A,C,F,G,H,I,J,L,M) / (B,D,E,K,N,O); Mecanismo=(a,c,f,g,h,i,j,l,m) / (b,d,e,k,n,o)</t>
+          <t>Alcance=(A) / (B); Mecanismo=(∅) / (b)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0,3910316228866577</t>
+          <t>0,25</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0,34896183013916016</t>
+          <t>0,1875</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0,7399934530258179</t>
+          <t>0,4375</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1,178239345550537</t>
+          <t>0,5563821792602539</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>
@@ -824,37 +906,45 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>101</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Alcance=(A,B,D,E,F,H,J,K,N,O) / (C,G,I,L,M); Mecanismo=(b,d,e,f,h,j,k,n,o) / (c,g,i,l,m)</t>
+          <t>Alcance=(A) / (B); Mecanismo=(a,c) / (∅)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0,3207746744155884</t>
+          <t>0,25</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0,2927582859992981</t>
+          <t>0,1875</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0,6135329604148865</t>
+          <t>0,4375</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0,9671359062194824</t>
+          <t>0,50819993019104</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>GeoMIP</t>
         </is>
       </c>
     </row>

</xml_diff>